<commit_message>
feat: wage groups update with rates
</commit_message>
<xml_diff>
--- a/input/202550 Kloklijst Padifood Flexspecialisten.xlsx
+++ b/input/202550 Kloklijst Padifood Flexspecialisten.xlsx
@@ -1,22 +1,58 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://padifoodoss.sharepoint.com/sites/hr/Gedeelde documenten/General/Administratie HR/Urenregistratie/1. Kloklijsten uitzendbureaus/2. Flexspecialisten/2025/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tombe\Documents\Hammer\projects\26PAD1\padifood-backend\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EADE11F8-9B1E-441F-A511-3616D4015887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83252FBA-4E17-43B2-8F70-CF6377E51486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="unique_names" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -575,9 +611,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="hh:mm\+"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="hh:mm\+"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -591,61 +626,73 @@
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -711,7 +758,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -726,7 +773,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="20" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -744,7 +791,7 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -761,7 +808,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -777,7 +824,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1094,12 +1141,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R486"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="18" width="15.42578125" customWidth="1"/>
+    <col min="1" max="18" width="15.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="15.95" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1155,7 +1202,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>18</v>
       </c>
@@ -1211,7 +1258,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
         <v>19</v>
       </c>
@@ -1267,7 +1314,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
         <v>19</v>
       </c>
@@ -1323,7 +1370,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
         <v>19</v>
       </c>
@@ -1379,7 +1426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="6" t="s">
         <v>19</v>
       </c>
@@ -1435,7 +1482,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
         <v>19</v>
       </c>
@@ -1491,7 +1538,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="6" t="s">
         <v>19</v>
       </c>
@@ -1547,7 +1594,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
         <v>19</v>
       </c>
@@ -1603,7 +1650,7 @@
         <v>32.25</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
         <v>22</v>
       </c>
@@ -1659,7 +1706,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
         <v>19</v>
       </c>
@@ -1715,7 +1762,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="6" t="s">
         <v>19</v>
       </c>
@@ -1771,7 +1818,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
         <v>19</v>
       </c>
@@ -1827,7 +1874,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="6" t="s">
         <v>19</v>
       </c>
@@ -1883,7 +1930,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
         <v>19</v>
       </c>
@@ -1939,7 +1986,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="6" t="s">
         <v>19</v>
       </c>
@@ -1995,7 +2042,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
         <v>19</v>
       </c>
@@ -2051,7 +2098,7 @@
         <v>40.25</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="6" t="s">
         <v>26</v>
       </c>
@@ -2107,7 +2154,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
         <v>19</v>
       </c>
@@ -2163,7 +2210,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="6" t="s">
         <v>19</v>
       </c>
@@ -2219,7 +2266,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="s">
         <v>19</v>
       </c>
@@ -2275,7 +2322,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="6" t="s">
         <v>19</v>
       </c>
@@ -2331,7 +2378,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="6" t="s">
         <v>19</v>
       </c>
@@ -2387,7 +2434,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A24" s="6" t="s">
         <v>19</v>
       </c>
@@ -2443,7 +2490,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A25" s="6" t="s">
         <v>19</v>
       </c>
@@ -2499,7 +2546,7 @@
         <v>36.75</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="6" t="s">
         <v>29</v>
       </c>
@@ -2555,7 +2602,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A27" s="6" t="s">
         <v>19</v>
       </c>
@@ -2611,7 +2658,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="6" t="s">
         <v>19</v>
       </c>
@@ -2667,7 +2714,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A29" s="6" t="s">
         <v>19</v>
       </c>
@@ -2723,7 +2770,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A30" s="6" t="s">
         <v>19</v>
       </c>
@@ -2779,7 +2826,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A31" s="6" t="s">
         <v>19</v>
       </c>
@@ -2835,7 +2882,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A32" s="6" t="s">
         <v>19</v>
       </c>
@@ -2891,7 +2938,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" s="6" t="s">
         <v>19</v>
       </c>
@@ -2947,7 +2994,7 @@
         <v>42.5</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A34" s="6" t="s">
         <v>19</v>
       </c>
@@ -3003,7 +3050,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" s="6" t="s">
         <v>19</v>
       </c>
@@ -3059,7 +3106,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" s="6" t="s">
         <v>19</v>
       </c>
@@ -3115,7 +3162,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" s="6" t="s">
         <v>19</v>
       </c>
@@ -3171,7 +3218,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" s="6" t="s">
         <v>19</v>
       </c>
@@ -3227,7 +3274,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="39" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" s="6" t="s">
         <v>19</v>
       </c>
@@ -3283,7 +3330,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A40" s="6" t="s">
         <v>19</v>
       </c>
@@ -3339,7 +3386,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A41" s="6" t="s">
         <v>19</v>
       </c>
@@ -3395,7 +3442,7 @@
         <v>31.5</v>
       </c>
     </row>
-    <row r="42" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A42" s="6" t="s">
         <v>35</v>
       </c>
@@ -3451,7 +3498,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" s="6" t="s">
         <v>19</v>
       </c>
@@ -3507,7 +3554,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" s="6" t="s">
         <v>19</v>
       </c>
@@ -3563,7 +3610,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A45" s="6" t="s">
         <v>19</v>
       </c>
@@ -3619,7 +3666,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" s="6" t="s">
         <v>19</v>
       </c>
@@ -3675,7 +3722,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A47" s="6" t="s">
         <v>19</v>
       </c>
@@ -3731,7 +3778,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A48" s="6" t="s">
         <v>19</v>
       </c>
@@ -3787,7 +3834,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A49" s="6" t="s">
         <v>19</v>
       </c>
@@ -3843,7 +3890,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="50" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" s="6" t="s">
         <v>19</v>
       </c>
@@ -3899,7 +3946,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="51" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" s="6" t="s">
         <v>19</v>
       </c>
@@ -3955,7 +4002,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="52" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" s="6" t="s">
         <v>19</v>
       </c>
@@ -4011,7 +4058,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="53" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A53" s="6" t="s">
         <v>19</v>
       </c>
@@ -4067,7 +4114,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A54" s="6" t="s">
         <v>19</v>
       </c>
@@ -4123,7 +4170,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="55" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" s="6" t="s">
         <v>19</v>
       </c>
@@ -4179,7 +4226,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="56" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A56" s="6" t="s">
         <v>19</v>
       </c>
@@ -4235,7 +4282,7 @@
         <v>41.25</v>
       </c>
     </row>
-    <row r="57" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A57" s="6" t="s">
         <v>41</v>
       </c>
@@ -4291,7 +4338,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="58" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A58" s="6" t="s">
         <v>19</v>
       </c>
@@ -4347,7 +4394,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="59" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" s="6" t="s">
         <v>19</v>
       </c>
@@ -4403,7 +4450,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A60" s="6" t="s">
         <v>19</v>
       </c>
@@ -4459,7 +4506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A61" s="6" t="s">
         <v>19</v>
       </c>
@@ -4515,7 +4562,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="62" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" s="6" t="s">
         <v>19</v>
       </c>
@@ -4571,7 +4618,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A63" s="6" t="s">
         <v>19</v>
       </c>
@@ -4627,7 +4674,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="64" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A64" s="6" t="s">
         <v>19</v>
       </c>
@@ -4683,7 +4730,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="65" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A65" s="6" t="s">
         <v>44</v>
       </c>
@@ -4739,7 +4786,7 @@
         <v>3.25</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" s="6" t="s">
         <v>19</v>
       </c>
@@ -4795,7 +4842,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" s="6" t="s">
         <v>19</v>
       </c>
@@ -4851,7 +4898,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="68" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" s="6" t="s">
         <v>19</v>
       </c>
@@ -4907,7 +4954,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" s="6" t="s">
         <v>19</v>
       </c>
@@ -4963,7 +5010,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A70" s="6" t="s">
         <v>19</v>
       </c>
@@ -5019,7 +5066,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="71" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A71" s="6" t="s">
         <v>19</v>
       </c>
@@ -5075,7 +5122,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="72" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="6" t="s">
         <v>19</v>
       </c>
@@ -5131,7 +5178,7 @@
         <v>3.25</v>
       </c>
     </row>
-    <row r="73" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="6" t="s">
         <v>46</v>
       </c>
@@ -5187,7 +5234,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="74" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="6" t="s">
         <v>19</v>
       </c>
@@ -5243,7 +5290,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="6" t="s">
         <v>19</v>
       </c>
@@ -5299,7 +5346,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="6" t="s">
         <v>19</v>
       </c>
@@ -5355,7 +5402,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="77" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A77" s="6" t="s">
         <v>19</v>
       </c>
@@ -5411,7 +5458,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="6" t="s">
         <v>19</v>
       </c>
@@ -5467,7 +5514,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="79" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" s="6" t="s">
         <v>19</v>
       </c>
@@ -5523,7 +5570,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="80" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="6" t="s">
         <v>19</v>
       </c>
@@ -5579,7 +5626,7 @@
         <v>30.25</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="6" t="s">
         <v>49</v>
       </c>
@@ -5635,7 +5682,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="82" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A82" s="6" t="s">
         <v>19</v>
       </c>
@@ -5691,7 +5738,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="83" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A83" s="6" t="s">
         <v>19</v>
       </c>
@@ -5747,7 +5794,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A84" s="6" t="s">
         <v>19</v>
       </c>
@@ -5803,7 +5850,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="85" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A85" s="6" t="s">
         <v>19</v>
       </c>
@@ -5859,7 +5906,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" s="6" t="s">
         <v>19</v>
       </c>
@@ -5915,7 +5962,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A87" s="6" t="s">
         <v>19</v>
       </c>
@@ -5971,7 +6018,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="88" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A88" s="6" t="s">
         <v>19</v>
       </c>
@@ -6027,7 +6074,7 @@
         <v>39.5</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" s="6" t="s">
         <v>52</v>
       </c>
@@ -6083,7 +6130,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A90" s="6" t="s">
         <v>19</v>
       </c>
@@ -6139,7 +6186,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A91" s="6" t="s">
         <v>19</v>
       </c>
@@ -6195,7 +6242,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A92" s="6" t="s">
         <v>19</v>
       </c>
@@ -6251,7 +6298,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="93" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A93" s="6" t="s">
         <v>19</v>
       </c>
@@ -6307,7 +6354,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A94" s="6" t="s">
         <v>19</v>
       </c>
@@ -6363,7 +6410,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A95" s="6" t="s">
         <v>19</v>
       </c>
@@ -6419,7 +6466,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="96" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A96" s="6" t="s">
         <v>19</v>
       </c>
@@ -6475,7 +6522,7 @@
         <v>41.25</v>
       </c>
     </row>
-    <row r="97" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A97" s="6" t="s">
         <v>55</v>
       </c>
@@ -6531,7 +6578,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A98" s="6" t="s">
         <v>19</v>
       </c>
@@ -6587,7 +6634,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A99" s="6" t="s">
         <v>19</v>
       </c>
@@ -6643,7 +6690,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A100" s="6" t="s">
         <v>19</v>
       </c>
@@ -6699,7 +6746,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="101" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="6" t="s">
         <v>19</v>
       </c>
@@ -6755,7 +6802,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="102" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A102" s="6" t="s">
         <v>19</v>
       </c>
@@ -6811,7 +6858,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="103" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A103" s="6" t="s">
         <v>19</v>
       </c>
@@ -6867,7 +6914,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A104" s="6" t="s">
         <v>59</v>
       </c>
@@ -6923,7 +6970,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A105" s="6" t="s">
         <v>19</v>
       </c>
@@ -6979,7 +7026,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A106" s="6" t="s">
         <v>19</v>
       </c>
@@ -7035,7 +7082,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A107" s="6" t="s">
         <v>19</v>
       </c>
@@ -7091,7 +7138,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="108" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A108" s="6" t="s">
         <v>19</v>
       </c>
@@ -7147,7 +7194,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="109" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A109" s="6" t="s">
         <v>19</v>
       </c>
@@ -7203,7 +7250,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="110" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A110" s="6" t="s">
         <v>19</v>
       </c>
@@ -7259,7 +7306,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A111" s="6" t="s">
         <v>19</v>
       </c>
@@ -7315,7 +7362,7 @@
         <v>27.5</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A112" s="6" t="s">
         <v>61</v>
       </c>
@@ -7371,7 +7418,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A113" s="6" t="s">
         <v>19</v>
       </c>
@@ -7427,7 +7474,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A114" s="6" t="s">
         <v>19</v>
       </c>
@@ -7483,7 +7530,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A115" s="6" t="s">
         <v>19</v>
       </c>
@@ -7539,7 +7586,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A116" s="6" t="s">
         <v>19</v>
       </c>
@@ -7595,7 +7642,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="117" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A117" s="6" t="s">
         <v>19</v>
       </c>
@@ -7651,7 +7698,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A118" s="6" t="s">
         <v>19</v>
       </c>
@@ -7707,7 +7754,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="119" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A119" s="6" t="s">
         <v>19</v>
       </c>
@@ -7763,7 +7810,7 @@
         <v>42.5</v>
       </c>
     </row>
-    <row r="120" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A120" s="6" t="s">
         <v>65</v>
       </c>
@@ -7819,7 +7866,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="121" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A121" s="6" t="s">
         <v>19</v>
       </c>
@@ -7875,7 +7922,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="122" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A122" s="6" t="s">
         <v>19</v>
       </c>
@@ -7931,7 +7978,7 @@
         <v>10.25</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="6" t="s">
         <v>19</v>
       </c>
@@ -7987,7 +8034,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="6" t="s">
         <v>19</v>
       </c>
@@ -8043,7 +8090,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="125" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A125" s="6" t="s">
         <v>19</v>
       </c>
@@ -8099,7 +8146,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A126" s="6" t="s">
         <v>19</v>
       </c>
@@ -8155,7 +8202,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="127" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A127" s="6" t="s">
         <v>19</v>
       </c>
@@ -8211,7 +8258,7 @@
         <v>44.25</v>
       </c>
     </row>
-    <row r="128" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A128" s="6" t="s">
         <v>19</v>
       </c>
@@ -8267,7 +8314,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="129" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A129" s="6" t="s">
         <v>19</v>
       </c>
@@ -8323,7 +8370,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="130" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A130" s="6" t="s">
         <v>19</v>
       </c>
@@ -8379,7 +8426,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A131" s="6" t="s">
         <v>19</v>
       </c>
@@ -8435,7 +8482,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="132" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A132" s="6" t="s">
         <v>19</v>
       </c>
@@ -8491,7 +8538,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="133" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A133" s="6" t="s">
         <v>19</v>
       </c>
@@ -8547,7 +8594,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A134" s="6" t="s">
         <v>19</v>
       </c>
@@ -8603,7 +8650,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A135" s="6" t="s">
         <v>29</v>
       </c>
@@ -8659,7 +8706,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A136" s="6" t="s">
         <v>19</v>
       </c>
@@ -8715,7 +8762,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="137" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A137" s="6" t="s">
         <v>19</v>
       </c>
@@ -8771,7 +8818,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A138" s="6" t="s">
         <v>19</v>
       </c>
@@ -8827,7 +8874,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A139" s="6" t="s">
         <v>19</v>
       </c>
@@ -8883,7 +8930,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="140" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A140" s="6" t="s">
         <v>19</v>
       </c>
@@ -8939,7 +8986,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="141" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A141" s="6" t="s">
         <v>19</v>
       </c>
@@ -8995,7 +9042,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="142" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A142" s="6" t="s">
         <v>72</v>
       </c>
@@ -9051,7 +9098,7 @@
         <v>5.25</v>
       </c>
     </row>
-    <row r="143" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A143" s="6" t="s">
         <v>19</v>
       </c>
@@ -9107,7 +9154,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="144" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A144" s="6" t="s">
         <v>19</v>
       </c>
@@ -9163,7 +9210,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="145" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A145" s="6" t="s">
         <v>19</v>
       </c>
@@ -9219,7 +9266,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="146" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A146" s="6" t="s">
         <v>19</v>
       </c>
@@ -9275,7 +9322,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="147" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A147" s="6" t="s">
         <v>19</v>
       </c>
@@ -9331,7 +9378,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="148" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A148" s="6" t="s">
         <v>19</v>
       </c>
@@ -9387,7 +9434,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="149" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A149" s="6" t="s">
         <v>19</v>
       </c>
@@ -9443,7 +9490,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="150" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A150" s="6" t="s">
         <v>74</v>
       </c>
@@ -9499,7 +9546,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="151" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A151" s="6" t="s">
         <v>19</v>
       </c>
@@ -9555,7 +9602,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="152" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A152" s="6" t="s">
         <v>19</v>
       </c>
@@ -9611,7 +9658,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="153" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A153" s="6" t="s">
         <v>19</v>
       </c>
@@ -9667,7 +9714,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="154" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A154" s="6" t="s">
         <v>19</v>
       </c>
@@ -9723,7 +9770,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="155" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A155" s="6" t="s">
         <v>19</v>
       </c>
@@ -9779,7 +9826,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="156" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A156" s="6" t="s">
         <v>19</v>
       </c>
@@ -9835,7 +9882,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="157" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A157" s="6" t="s">
         <v>19</v>
       </c>
@@ -9891,7 +9938,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="158" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A158" s="6" t="s">
         <v>77</v>
       </c>
@@ -9947,7 +9994,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="159" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A159" s="6" t="s">
         <v>19</v>
       </c>
@@ -10003,7 +10050,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="160" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A160" s="6" t="s">
         <v>19</v>
       </c>
@@ -10059,7 +10106,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="161" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A161" s="6" t="s">
         <v>19</v>
       </c>
@@ -10115,7 +10162,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="162" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A162" s="6" t="s">
         <v>19</v>
       </c>
@@ -10171,7 +10218,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="163" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A163" s="6" t="s">
         <v>19</v>
       </c>
@@ -10227,7 +10274,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="164" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A164" s="6" t="s">
         <v>19</v>
       </c>
@@ -10283,7 +10330,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="165" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A165" s="6" t="s">
         <v>19</v>
       </c>
@@ -10339,7 +10386,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="166" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A166" s="6" t="s">
         <v>80</v>
       </c>
@@ -10395,7 +10442,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="167" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A167" s="6" t="s">
         <v>19</v>
       </c>
@@ -10451,7 +10498,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="168" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A168" s="6" t="s">
         <v>19</v>
       </c>
@@ -10507,7 +10554,7 @@
         <v>9.75</v>
       </c>
     </row>
-    <row r="169" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A169" s="6" t="s">
         <v>19</v>
       </c>
@@ -10563,7 +10610,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="170" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A170" s="6" t="s">
         <v>19</v>
       </c>
@@ -10619,7 +10666,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="171" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A171" s="6" t="s">
         <v>19</v>
       </c>
@@ -10675,7 +10722,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="172" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A172" s="6" t="s">
         <v>19</v>
       </c>
@@ -10731,7 +10778,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="173" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A173" s="6" t="s">
         <v>19</v>
       </c>
@@ -10787,7 +10834,7 @@
         <v>43.25</v>
       </c>
     </row>
-    <row r="174" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A174" s="6" t="s">
         <v>83</v>
       </c>
@@ -10843,7 +10890,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="175" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A175" s="6" t="s">
         <v>19</v>
       </c>
@@ -10899,7 +10946,7 @@
         <v>6.25</v>
       </c>
     </row>
-    <row r="176" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A176" s="6" t="s">
         <v>19</v>
       </c>
@@ -10955,7 +11002,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="177" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A177" s="6" t="s">
         <v>19</v>
       </c>
@@ -11011,7 +11058,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="178" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A178" s="6" t="s">
         <v>19</v>
       </c>
@@ -11067,7 +11114,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="179" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A179" s="6" t="s">
         <v>19</v>
       </c>
@@ -11123,7 +11170,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="180" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A180" s="6" t="s">
         <v>19</v>
       </c>
@@ -11179,7 +11226,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="181" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A181" s="6" t="s">
         <v>19</v>
       </c>
@@ -11235,7 +11282,7 @@
         <v>34.5</v>
       </c>
     </row>
-    <row r="182" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A182" s="6" t="s">
         <v>86</v>
       </c>
@@ -11291,7 +11338,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="183" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A183" s="6" t="s">
         <v>19</v>
       </c>
@@ -11347,7 +11394,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="184" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A184" s="6" t="s">
         <v>19</v>
       </c>
@@ -11403,7 +11450,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="185" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A185" s="6" t="s">
         <v>19</v>
       </c>
@@ -11459,7 +11506,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="186" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A186" s="6" t="s">
         <v>19</v>
       </c>
@@ -11515,7 +11562,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="187" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A187" s="6" t="s">
         <v>19</v>
       </c>
@@ -11571,7 +11618,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="188" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A188" s="6" t="s">
         <v>19</v>
       </c>
@@ -11627,7 +11674,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="189" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A189" s="6" t="s">
         <v>19</v>
       </c>
@@ -11683,7 +11730,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="190" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A190" s="6" t="s">
         <v>90</v>
       </c>
@@ -11739,7 +11786,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="191" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A191" s="6" t="s">
         <v>19</v>
       </c>
@@ -11795,7 +11842,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="192" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A192" s="6" t="s">
         <v>19</v>
       </c>
@@ -11851,7 +11898,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="193" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A193" s="6" t="s">
         <v>19</v>
       </c>
@@ -11907,7 +11954,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="194" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A194" s="6" t="s">
         <v>19</v>
       </c>
@@ -11963,7 +12010,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="195" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A195" s="6" t="s">
         <v>19</v>
       </c>
@@ -12019,7 +12066,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="196" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A196" s="6" t="s">
         <v>19</v>
       </c>
@@ -12075,7 +12122,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="197" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A197" s="6" t="s">
         <v>19</v>
       </c>
@@ -12131,7 +12178,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="198" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A198" s="6" t="s">
         <v>93</v>
       </c>
@@ -12187,7 +12234,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="199" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A199" s="6" t="s">
         <v>19</v>
       </c>
@@ -12243,7 +12290,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="200" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A200" s="6" t="s">
         <v>19</v>
       </c>
@@ -12299,7 +12346,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="201" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A201" s="6" t="s">
         <v>19</v>
       </c>
@@ -12355,7 +12402,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="202" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A202" s="6" t="s">
         <v>19</v>
       </c>
@@ -12411,7 +12458,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="203" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A203" s="6" t="s">
         <v>19</v>
       </c>
@@ -12467,7 +12514,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="204" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A204" s="6" t="s">
         <v>19</v>
       </c>
@@ -12523,7 +12570,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="205" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A205" s="6" t="s">
         <v>96</v>
       </c>
@@ -12579,7 +12626,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="206" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A206" s="6" t="s">
         <v>19</v>
       </c>
@@ -12635,7 +12682,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="207" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A207" s="6" t="s">
         <v>19</v>
       </c>
@@ -12691,7 +12738,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="208" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A208" s="6" t="s">
         <v>19</v>
       </c>
@@ -12747,7 +12794,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="209" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A209" s="6" t="s">
         <v>19</v>
       </c>
@@ -12803,7 +12850,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="210" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A210" s="6" t="s">
         <v>19</v>
       </c>
@@ -12859,7 +12906,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="211" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A211" s="6" t="s">
         <v>19</v>
       </c>
@@ -12915,7 +12962,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="212" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A212" s="6" t="s">
         <v>19</v>
       </c>
@@ -12971,7 +13018,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="213" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A213" s="6" t="s">
         <v>99</v>
       </c>
@@ -13027,7 +13074,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="214" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A214" s="6" t="s">
         <v>19</v>
       </c>
@@ -13083,7 +13130,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="215" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A215" s="6" t="s">
         <v>19</v>
       </c>
@@ -13139,7 +13186,7 @@
         <v>6.25</v>
       </c>
     </row>
-    <row r="216" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A216" s="6" t="s">
         <v>19</v>
       </c>
@@ -13195,7 +13242,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="217" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A217" s="6" t="s">
         <v>19</v>
       </c>
@@ -13251,7 +13298,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="218" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A218" s="6" t="s">
         <v>19</v>
       </c>
@@ -13307,7 +13354,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="219" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A219" s="6" t="s">
         <v>19</v>
       </c>
@@ -13363,7 +13410,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="220" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A220" s="6" t="s">
         <v>19</v>
       </c>
@@ -13419,7 +13466,7 @@
         <v>38.5</v>
       </c>
     </row>
-    <row r="221" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A221" s="6" t="s">
         <v>102</v>
       </c>
@@ -13475,7 +13522,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="222" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A222" s="6" t="s">
         <v>102</v>
       </c>
@@ -13531,7 +13578,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="223" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A223" s="6" t="s">
         <v>19</v>
       </c>
@@ -13587,7 +13634,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="224" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A224" s="6" t="s">
         <v>19</v>
       </c>
@@ -13643,7 +13690,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="225" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A225" s="6" t="s">
         <v>19</v>
       </c>
@@ -13699,7 +13746,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="226" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A226" s="6" t="s">
         <v>19</v>
       </c>
@@ -13755,7 +13802,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="227" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A227" s="6" t="s">
         <v>19</v>
       </c>
@@ -13811,7 +13858,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="228" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A228" s="6" t="s">
         <v>104</v>
       </c>
@@ -13867,7 +13914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A229" s="6" t="s">
         <v>19</v>
       </c>
@@ -13923,7 +13970,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="230" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A230" s="6" t="s">
         <v>19</v>
       </c>
@@ -13979,7 +14026,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="231" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A231" s="6" t="s">
         <v>19</v>
       </c>
@@ -14035,7 +14082,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="232" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A232" s="6" t="s">
         <v>19</v>
       </c>
@@ -14091,7 +14138,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="233" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A233" s="6" t="s">
         <v>19</v>
       </c>
@@ -14147,7 +14194,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="234" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A234" s="6" t="s">
         <v>19</v>
       </c>
@@ -14203,7 +14250,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="235" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A235" s="6" t="s">
         <v>19</v>
       </c>
@@ -14259,7 +14306,7 @@
         <v>29.5</v>
       </c>
     </row>
-    <row r="236" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A236" s="6" t="s">
         <v>107</v>
       </c>
@@ -14315,7 +14362,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="237" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A237" s="6" t="s">
         <v>19</v>
       </c>
@@ -14371,7 +14418,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="238" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A238" s="6" t="s">
         <v>19</v>
       </c>
@@ -14427,7 +14474,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="239" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A239" s="6" t="s">
         <v>19</v>
       </c>
@@ -14483,7 +14530,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="240" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A240" s="6" t="s">
         <v>19</v>
       </c>
@@ -14539,7 +14586,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="241" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A241" s="6" t="s">
         <v>19</v>
       </c>
@@ -14595,7 +14642,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="242" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A242" s="6" t="s">
         <v>19</v>
       </c>
@@ -14651,7 +14698,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="243" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A243" s="6" t="s">
         <v>19</v>
       </c>
@@ -14707,7 +14754,7 @@
         <v>28.5</v>
       </c>
     </row>
-    <row r="244" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A244" s="6" t="s">
         <v>110</v>
       </c>
@@ -14763,7 +14810,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="245" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A245" s="6" t="s">
         <v>19</v>
       </c>
@@ -14819,7 +14866,7 @@
         <v>6.25</v>
       </c>
     </row>
-    <row r="246" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A246" s="6" t="s">
         <v>19</v>
       </c>
@@ -14875,7 +14922,7 @@
         <v>3.75</v>
       </c>
     </row>
-    <row r="247" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A247" s="6" t="s">
         <v>19</v>
       </c>
@@ -14931,7 +14978,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="248" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A248" s="6" t="s">
         <v>19</v>
       </c>
@@ -14987,7 +15034,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="249" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A249" s="6" t="s">
         <v>19</v>
       </c>
@@ -15043,7 +15090,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="250" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A250" s="6" t="s">
         <v>19</v>
       </c>
@@ -15099,7 +15146,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="251" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A251" s="6" t="s">
         <v>19</v>
       </c>
@@ -15155,7 +15202,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="252" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A252" s="6" t="s">
         <v>112</v>
       </c>
@@ -15211,7 +15258,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="253" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A253" s="6" t="s">
         <v>19</v>
       </c>
@@ -15267,7 +15314,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="254" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A254" s="6" t="s">
         <v>19</v>
       </c>
@@ -15323,7 +15370,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="255" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A255" s="6" t="s">
         <v>19</v>
       </c>
@@ -15379,7 +15426,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="256" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A256" s="6" t="s">
         <v>19</v>
       </c>
@@ -15435,7 +15482,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="257" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A257" s="6" t="s">
         <v>19</v>
       </c>
@@ -15491,7 +15538,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="258" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A258" s="6" t="s">
         <v>19</v>
       </c>
@@ -15547,7 +15594,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="259" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A259" s="6" t="s">
         <v>19</v>
       </c>
@@ -15603,7 +15650,7 @@
         <v>33.5</v>
       </c>
     </row>
-    <row r="260" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A260" s="6" t="s">
         <v>116</v>
       </c>
@@ -15659,7 +15706,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="261" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A261" s="6" t="s">
         <v>19</v>
       </c>
@@ -15715,7 +15762,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="262" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A262" s="6" t="s">
         <v>19</v>
       </c>
@@ -15771,7 +15818,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="263" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A263" s="6" t="s">
         <v>19</v>
       </c>
@@ -15827,7 +15874,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="264" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A264" s="6" t="s">
         <v>19</v>
       </c>
@@ -15883,7 +15930,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="265" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A265" s="6" t="s">
         <v>19</v>
       </c>
@@ -15939,7 +15986,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="266" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A266" s="6" t="s">
         <v>19</v>
       </c>
@@ -15995,7 +16042,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="267" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A267" s="6" t="s">
         <v>19</v>
       </c>
@@ -16051,7 +16098,7 @@
         <v>38.5</v>
       </c>
     </row>
-    <row r="268" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A268" s="6" t="s">
         <v>119</v>
       </c>
@@ -16107,7 +16154,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="269" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A269" s="6" t="s">
         <v>19</v>
       </c>
@@ -16163,7 +16210,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="270" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A270" s="6" t="s">
         <v>19</v>
       </c>
@@ -16219,7 +16266,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="271" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A271" s="6" t="s">
         <v>19</v>
       </c>
@@ -16275,7 +16322,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="272" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A272" s="6" t="s">
         <v>19</v>
       </c>
@@ -16331,7 +16378,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="273" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A273" s="6" t="s">
         <v>19</v>
       </c>
@@ -16387,7 +16434,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="274" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A274" s="6" t="s">
         <v>19</v>
       </c>
@@ -16443,7 +16490,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="275" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A275" s="6" t="s">
         <v>19</v>
       </c>
@@ -16499,7 +16546,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="276" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A276" s="6" t="s">
         <v>122</v>
       </c>
@@ -16555,7 +16602,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="277" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A277" s="6" t="s">
         <v>19</v>
       </c>
@@ -16611,7 +16658,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="278" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A278" s="6" t="s">
         <v>19</v>
       </c>
@@ -16667,7 +16714,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="279" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A279" s="6" t="s">
         <v>19</v>
       </c>
@@ -16723,7 +16770,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="280" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A280" s="6" t="s">
         <v>19</v>
       </c>
@@ -16779,7 +16826,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="281" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A281" s="6" t="s">
         <v>19</v>
       </c>
@@ -16835,7 +16882,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="282" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A282" s="6" t="s">
         <v>19</v>
       </c>
@@ -16891,7 +16938,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="283" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A283" s="6" t="s">
         <v>19</v>
       </c>
@@ -16947,7 +16994,7 @@
         <v>35.75</v>
       </c>
     </row>
-    <row r="284" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A284" s="6" t="s">
         <v>19</v>
       </c>
@@ -17003,7 +17050,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="285" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A285" s="6" t="s">
         <v>19</v>
       </c>
@@ -17059,7 +17106,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="286" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A286" s="6" t="s">
         <v>19</v>
       </c>
@@ -17115,7 +17162,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="287" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A287" s="6" t="s">
         <v>19</v>
       </c>
@@ -17171,7 +17218,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="288" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A288" s="6" t="s">
         <v>19</v>
       </c>
@@ -17227,7 +17274,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="289" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A289" s="6" t="s">
         <v>19</v>
       </c>
@@ -17283,7 +17330,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="290" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A290" s="6" t="s">
         <v>19</v>
       </c>
@@ -17339,7 +17386,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="291" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A291" s="6" t="s">
         <v>19</v>
       </c>
@@ -17395,7 +17442,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="292" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A292" s="6" t="s">
         <v>19</v>
       </c>
@@ -17451,7 +17498,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="293" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A293" s="6" t="s">
         <v>19</v>
       </c>
@@ -17507,7 +17554,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="294" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A294" s="6" t="s">
         <v>19</v>
       </c>
@@ -17563,7 +17610,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="295" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A295" s="6" t="s">
         <v>19</v>
       </c>
@@ -17619,7 +17666,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="296" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A296" s="6" t="s">
         <v>19</v>
       </c>
@@ -17675,7 +17722,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="297" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A297" s="6" t="s">
         <v>19</v>
       </c>
@@ -17731,7 +17778,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="298" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A298" s="6" t="s">
         <v>19</v>
       </c>
@@ -17787,7 +17834,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="299" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A299" s="6" t="s">
         <v>19</v>
       </c>
@@ -17843,7 +17890,7 @@
         <v>38.75</v>
       </c>
     </row>
-    <row r="300" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A300" s="6" t="s">
         <v>127</v>
       </c>
@@ -17899,7 +17946,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="301" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A301" s="6" t="s">
         <v>19</v>
       </c>
@@ -17955,7 +18002,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="302" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A302" s="6" t="s">
         <v>19</v>
       </c>
@@ -18011,7 +18058,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="303" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A303" s="6" t="s">
         <v>19</v>
       </c>
@@ -18067,7 +18114,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="304" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A304" s="6" t="s">
         <v>19</v>
       </c>
@@ -18123,7 +18170,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="305" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A305" s="6" t="s">
         <v>19</v>
       </c>
@@ -18179,7 +18226,7 @@
         <v>4.75</v>
       </c>
     </row>
-    <row r="306" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A306" s="6" t="s">
         <v>19</v>
       </c>
@@ -18235,7 +18282,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="307" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A307" s="6" t="s">
         <v>19</v>
       </c>
@@ -18291,7 +18338,7 @@
         <v>48.5</v>
       </c>
     </row>
-    <row r="308" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A308" s="6" t="s">
         <v>19</v>
       </c>
@@ -18347,7 +18394,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="309" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A309" s="6" t="s">
         <v>19</v>
       </c>
@@ -18403,7 +18450,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="310" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A310" s="6" t="s">
         <v>19</v>
       </c>
@@ -18459,7 +18506,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="311" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A311" s="6" t="s">
         <v>19</v>
       </c>
@@ -18515,7 +18562,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="312" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A312" s="6" t="s">
         <v>19</v>
       </c>
@@ -18571,7 +18618,7 @@
         <v>9.25</v>
       </c>
     </row>
-    <row r="313" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A313" s="6" t="s">
         <v>19</v>
       </c>
@@ -18627,7 +18674,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="314" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A314" s="6" t="s">
         <v>19</v>
       </c>
@@ -18683,7 +18730,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="315" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A315" s="6" t="s">
         <v>19</v>
       </c>
@@ -18739,7 +18786,7 @@
         <v>43.5</v>
       </c>
     </row>
-    <row r="316" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A316" s="6" t="s">
         <v>132</v>
       </c>
@@ -18795,7 +18842,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="317" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A317" s="6" t="s">
         <v>19</v>
       </c>
@@ -18851,7 +18898,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="318" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A318" s="6" t="s">
         <v>19</v>
       </c>
@@ -18907,7 +18954,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="319" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A319" s="6" t="s">
         <v>19</v>
       </c>
@@ -18963,7 +19010,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="320" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A320" s="6" t="s">
         <v>19</v>
       </c>
@@ -19019,7 +19066,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="321" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A321" s="6" t="s">
         <v>19</v>
       </c>
@@ -19075,7 +19122,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="322" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A322" s="6" t="s">
         <v>19</v>
       </c>
@@ -19131,7 +19178,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="323" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A323" s="6" t="s">
         <v>72</v>
       </c>
@@ -19187,7 +19234,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="324" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A324" s="6" t="s">
         <v>19</v>
       </c>
@@ -19243,7 +19290,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="325" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A325" s="6" t="s">
         <v>19</v>
       </c>
@@ -19299,7 +19346,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="326" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A326" s="6" t="s">
         <v>19</v>
       </c>
@@ -19355,7 +19402,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="327" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A327" s="6" t="s">
         <v>19</v>
       </c>
@@ -19411,7 +19458,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="328" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A328" s="6" t="s">
         <v>19</v>
       </c>
@@ -19467,7 +19514,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="329" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A329" s="6" t="s">
         <v>19</v>
       </c>
@@ -19523,7 +19570,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="330" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A330" s="6" t="s">
         <v>19</v>
       </c>
@@ -19579,7 +19626,7 @@
         <v>27.75</v>
       </c>
     </row>
-    <row r="331" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A331" s="6" t="s">
         <v>136</v>
       </c>
@@ -19635,7 +19682,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="332" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A332" s="6" t="s">
         <v>19</v>
       </c>
@@ -19691,7 +19738,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="333" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A333" s="6" t="s">
         <v>19</v>
       </c>
@@ -19747,7 +19794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="334" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A334" s="6" t="s">
         <v>19</v>
       </c>
@@ -19803,7 +19850,7 @@
         <v>9.75</v>
       </c>
     </row>
-    <row r="335" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A335" s="6" t="s">
         <v>19</v>
       </c>
@@ -19859,7 +19906,7 @@
         <v>9.5</v>
       </c>
     </row>
-    <row r="336" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A336" s="6" t="s">
         <v>19</v>
       </c>
@@ -19915,7 +19962,7 @@
         <v>8.25</v>
       </c>
     </row>
-    <row r="337" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A337" s="6" t="s">
         <v>19</v>
       </c>
@@ -19971,7 +20018,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="338" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A338" s="6" t="s">
         <v>19</v>
       </c>
@@ -20027,7 +20074,7 @@
         <v>50.75</v>
       </c>
     </row>
-    <row r="339" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A339" s="6" t="s">
         <v>19</v>
       </c>
@@ -20083,7 +20130,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="340" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A340" s="6" t="s">
         <v>19</v>
       </c>
@@ -20139,7 +20186,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="341" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A341" s="6" t="s">
         <v>19</v>
       </c>
@@ -20195,7 +20242,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="342" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A342" s="6" t="s">
         <v>19</v>
       </c>
@@ -20251,7 +20298,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="343" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A343" s="6" t="s">
         <v>19</v>
       </c>
@@ -20307,7 +20354,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="344" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A344" s="6" t="s">
         <v>19</v>
       </c>
@@ -20363,7 +20410,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="345" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A345" s="6" t="s">
         <v>19</v>
       </c>
@@ -20419,7 +20466,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="346" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A346" s="6" t="s">
         <v>19</v>
       </c>
@@ -20475,7 +20522,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="347" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A347" s="6" t="s">
         <v>19</v>
       </c>
@@ -20531,7 +20578,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="348" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A348" s="6" t="s">
         <v>19</v>
       </c>
@@ -20587,7 +20634,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="349" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A349" s="6" t="s">
         <v>19</v>
       </c>
@@ -20643,7 +20690,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="350" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A350" s="6" t="s">
         <v>19</v>
       </c>
@@ -20699,7 +20746,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="351" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A351" s="6" t="s">
         <v>19</v>
       </c>
@@ -20755,7 +20802,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="352" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A352" s="6" t="s">
         <v>19</v>
       </c>
@@ -20811,7 +20858,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="353" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A353" s="6" t="s">
         <v>19</v>
       </c>
@@ -20867,7 +20914,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="354" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A354" s="6" t="s">
         <v>19</v>
       </c>
@@ -20923,7 +20970,7 @@
         <v>42.75</v>
       </c>
     </row>
-    <row r="355" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A355" s="6" t="s">
         <v>141</v>
       </c>
@@ -20979,7 +21026,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="356" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A356" s="6" t="s">
         <v>19</v>
       </c>
@@ -21035,7 +21082,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="357" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A357" s="6" t="s">
         <v>19</v>
       </c>
@@ -21091,7 +21138,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="358" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A358" s="6" t="s">
         <v>19</v>
       </c>
@@ -21147,7 +21194,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="359" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A359" s="6" t="s">
         <v>19</v>
       </c>
@@ -21203,7 +21250,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="360" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A360" s="6" t="s">
         <v>19</v>
       </c>
@@ -21259,7 +21306,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="361" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A361" s="6" t="s">
         <v>19</v>
       </c>
@@ -21315,7 +21362,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="362" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A362" s="6" t="s">
         <v>19</v>
       </c>
@@ -21371,7 +21418,7 @@
         <v>42.75</v>
       </c>
     </row>
-    <row r="363" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A363" s="6" t="s">
         <v>143</v>
       </c>
@@ -21427,7 +21474,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="364" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A364" s="6" t="s">
         <v>19</v>
       </c>
@@ -21483,7 +21530,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="365" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A365" s="6" t="s">
         <v>19</v>
       </c>
@@ -21539,7 +21586,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="366" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A366" s="6" t="s">
         <v>19</v>
       </c>
@@ -21595,7 +21642,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="367" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A367" s="6" t="s">
         <v>19</v>
       </c>
@@ -21651,7 +21698,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="368" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A368" s="6" t="s">
         <v>19</v>
       </c>
@@ -21707,7 +21754,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="369" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A369" s="6" t="s">
         <v>19</v>
       </c>
@@ -21763,7 +21810,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="370" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A370" s="6" t="s">
         <v>19</v>
       </c>
@@ -21819,7 +21866,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="371" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A371" s="6" t="s">
         <v>145</v>
       </c>
@@ -21875,7 +21922,7 @@
         <v>9.25</v>
       </c>
     </row>
-    <row r="372" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A372" s="6" t="s">
         <v>19</v>
       </c>
@@ -21931,7 +21978,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="373" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A373" s="6" t="s">
         <v>19</v>
       </c>
@@ -21987,7 +22034,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="374" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A374" s="6" t="s">
         <v>19</v>
       </c>
@@ -22043,7 +22090,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="375" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A375" s="6" t="s">
         <v>19</v>
       </c>
@@ -22099,7 +22146,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="376" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A376" s="6" t="s">
         <v>19</v>
       </c>
@@ -22155,7 +22202,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="377" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A377" s="6" t="s">
         <v>19</v>
       </c>
@@ -22211,7 +22258,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="378" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A378" s="6" t="s">
         <v>19</v>
       </c>
@@ -22267,7 +22314,7 @@
         <v>43.75</v>
       </c>
     </row>
-    <row r="379" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A379" s="6" t="s">
         <v>148</v>
       </c>
@@ -22323,7 +22370,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="380" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A380" s="6" t="s">
         <v>19</v>
       </c>
@@ -22379,7 +22426,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="381" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A381" s="6" t="s">
         <v>19</v>
       </c>
@@ -22435,7 +22482,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="382" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A382" s="6" t="s">
         <v>19</v>
       </c>
@@ -22491,7 +22538,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="383" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A383" s="6" t="s">
         <v>19</v>
       </c>
@@ -22547,7 +22594,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="384" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A384" s="6" t="s">
         <v>19</v>
       </c>
@@ -22603,7 +22650,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="385" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A385" s="6" t="s">
         <v>19</v>
       </c>
@@ -22659,7 +22706,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="386" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A386" s="6" t="s">
         <v>151</v>
       </c>
@@ -22715,7 +22762,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="387" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A387" s="6" t="s">
         <v>19</v>
       </c>
@@ -22771,7 +22818,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="388" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A388" s="6" t="s">
         <v>19</v>
       </c>
@@ -22827,7 +22874,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="389" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A389" s="6" t="s">
         <v>19</v>
       </c>
@@ -22883,7 +22930,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="390" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A390" s="6" t="s">
         <v>19</v>
       </c>
@@ -22939,7 +22986,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="391" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A391" s="6" t="s">
         <v>19</v>
       </c>
@@ -22995,7 +23042,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="392" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A392" s="6" t="s">
         <v>19</v>
       </c>
@@ -23051,7 +23098,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="393" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A393" s="6" t="s">
         <v>19</v>
       </c>
@@ -23107,7 +23154,7 @@
         <v>36.5</v>
       </c>
     </row>
-    <row r="394" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A394" s="6" t="s">
         <v>154</v>
       </c>
@@ -23163,7 +23210,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="395" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A395" s="6" t="s">
         <v>19</v>
       </c>
@@ -23219,7 +23266,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="396" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A396" s="6" t="s">
         <v>19</v>
       </c>
@@ -23275,7 +23322,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="397" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A397" s="6" t="s">
         <v>19</v>
       </c>
@@ -23331,7 +23378,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="398" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A398" s="6" t="s">
         <v>19</v>
       </c>
@@ -23387,7 +23434,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="399" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A399" s="6" t="s">
         <v>19</v>
       </c>
@@ -23443,7 +23490,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="400" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A400" s="6" t="s">
         <v>19</v>
       </c>
@@ -23499,7 +23546,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="401" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A401" s="6" t="s">
         <v>156</v>
       </c>
@@ -23555,7 +23602,7 @@
         <v>8.5</v>
       </c>
     </row>
-    <row r="402" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A402" s="6" t="s">
         <v>19</v>
       </c>
@@ -23611,7 +23658,7 @@
         <v>6.25</v>
       </c>
     </row>
-    <row r="403" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A403" s="6" t="s">
         <v>19</v>
       </c>
@@ -23667,7 +23714,7 @@
         <v>9.25</v>
       </c>
     </row>
-    <row r="404" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A404" s="6" t="s">
         <v>19</v>
       </c>
@@ -23723,7 +23770,7 @@
         <v>8.75</v>
       </c>
     </row>
-    <row r="405" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A405" s="6" t="s">
         <v>19</v>
       </c>
@@ -23779,7 +23826,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="406" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A406" s="6" t="s">
         <v>19</v>
       </c>
@@ -23835,7 +23882,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="407" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A407" s="6" t="s">
         <v>19</v>
       </c>
@@ -23891,7 +23938,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="408" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A408" s="6" t="s">
         <v>19</v>
       </c>
@@ -23947,7 +23994,7 @@
         <v>40.5</v>
       </c>
     </row>
-    <row r="409" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A409" s="6" t="s">
         <v>159</v>
       </c>
@@ -24003,7 +24050,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="410" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A410" s="6" t="s">
         <v>19</v>
       </c>
@@ -24059,7 +24106,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="411" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A411" s="6" t="s">
         <v>19</v>
       </c>
@@ -24115,7 +24162,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="412" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A412" s="6" t="s">
         <v>19</v>
       </c>
@@ -24171,7 +24218,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="413" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A413" s="6" t="s">
         <v>19</v>
       </c>
@@ -24227,7 +24274,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="414" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A414" s="6" t="s">
         <v>19</v>
       </c>
@@ -24283,7 +24330,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="415" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A415" s="6" t="s">
         <v>19</v>
       </c>
@@ -24339,7 +24386,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="416" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A416" s="6" t="s">
         <v>19</v>
       </c>
@@ -24395,7 +24442,7 @@
         <v>38.75</v>
       </c>
     </row>
-    <row r="417" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A417" s="6" t="s">
         <v>162</v>
       </c>
@@ -24451,7 +24498,7 @@
         <v>4.75</v>
       </c>
     </row>
-    <row r="418" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A418" s="6" t="s">
         <v>19</v>
       </c>
@@ -24507,7 +24554,7 @@
         <v>6.25</v>
       </c>
     </row>
-    <row r="419" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A419" s="6" t="s">
         <v>19</v>
       </c>
@@ -24563,7 +24610,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="420" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A420" s="6" t="s">
         <v>19</v>
       </c>
@@ -24619,7 +24666,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="421" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A421" s="6" t="s">
         <v>19</v>
       </c>
@@ -24675,7 +24722,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="422" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A422" s="6" t="s">
         <v>19</v>
       </c>
@@ -24731,7 +24778,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="423" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A423" s="6" t="s">
         <v>19</v>
       </c>
@@ -24787,7 +24834,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="424" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A424" s="6" t="s">
         <v>19</v>
       </c>
@@ -24843,7 +24890,7 @@
         <v>34.25</v>
       </c>
     </row>
-    <row r="425" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A425" s="6" t="s">
         <v>164</v>
       </c>
@@ -24899,7 +24946,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="426" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A426" s="6" t="s">
         <v>19</v>
       </c>
@@ -24955,7 +25002,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="427" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A427" s="6" t="s">
         <v>19</v>
       </c>
@@ -25011,7 +25058,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="428" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A428" s="6" t="s">
         <v>19</v>
       </c>
@@ -25067,7 +25114,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="429" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A429" s="6" t="s">
         <v>19</v>
       </c>
@@ -25123,7 +25170,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="430" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A430" s="6" t="s">
         <v>19</v>
       </c>
@@ -25179,7 +25226,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="431" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A431" s="6" t="s">
         <v>19</v>
       </c>
@@ -25235,7 +25282,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="432" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A432" s="6" t="s">
         <v>19</v>
       </c>
@@ -25291,7 +25338,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="433" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A433" s="6" t="s">
         <v>19</v>
       </c>
@@ -25347,7 +25394,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="434" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A434" s="6" t="s">
         <v>19</v>
       </c>
@@ -25403,7 +25450,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="435" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A435" s="6" t="s">
         <v>19</v>
       </c>
@@ -25459,7 +25506,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="436" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A436" s="6" t="s">
         <v>19</v>
       </c>
@@ -25515,7 +25562,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="437" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A437" s="6" t="s">
         <v>19</v>
       </c>
@@ -25571,7 +25618,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="438" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A438" s="6" t="s">
         <v>19</v>
       </c>
@@ -25627,7 +25674,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="439" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A439" s="6" t="s">
         <v>19</v>
       </c>
@@ -25683,7 +25730,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="440" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A440" s="6" t="s">
         <v>19</v>
       </c>
@@ -25739,7 +25786,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="441" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A441" s="6" t="s">
         <v>169</v>
       </c>
@@ -25795,7 +25842,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="442" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A442" s="6" t="s">
         <v>19</v>
       </c>
@@ -25851,7 +25898,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="443" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A443" s="6" t="s">
         <v>19</v>
       </c>
@@ -25907,7 +25954,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="444" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A444" s="6" t="s">
         <v>19</v>
       </c>
@@ -25963,7 +26010,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="445" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A445" s="6" t="s">
         <v>19</v>
       </c>
@@ -26019,7 +26066,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="446" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A446" s="6" t="s">
         <v>19</v>
       </c>
@@ -26075,7 +26122,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="447" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A447" s="6" t="s">
         <v>19</v>
       </c>
@@ -26131,7 +26178,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="448" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A448" s="6" t="s">
         <v>19</v>
       </c>
@@ -26187,7 +26234,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="449" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A449" s="6" t="s">
         <v>171</v>
       </c>
@@ -26243,7 +26290,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="450" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A450" s="6" t="s">
         <v>19</v>
       </c>
@@ -26299,7 +26346,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="451" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A451" s="6" t="s">
         <v>19</v>
       </c>
@@ -26355,7 +26402,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="452" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A452" s="6" t="s">
         <v>19</v>
       </c>
@@ -26411,7 +26458,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="453" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A453" s="6" t="s">
         <v>19</v>
       </c>
@@ -26467,7 +26514,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="454" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A454" s="6" t="s">
         <v>19</v>
       </c>
@@ -26523,7 +26570,7 @@
         <v>4.75</v>
       </c>
     </row>
-    <row r="455" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A455" s="6" t="s">
         <v>19</v>
       </c>
@@ -26579,7 +26626,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="456" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A456" s="6" t="s">
         <v>19</v>
       </c>
@@ -26635,7 +26682,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="457" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A457" s="6" t="s">
         <v>19</v>
       </c>
@@ -26691,7 +26738,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="458" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A458" s="6" t="s">
         <v>19</v>
       </c>
@@ -26747,7 +26794,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="459" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A459" s="6" t="s">
         <v>19</v>
       </c>
@@ -26803,7 +26850,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="460" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A460" s="6" t="s">
         <v>19</v>
       </c>
@@ -26859,7 +26906,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="461" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A461" s="6" t="s">
         <v>19</v>
       </c>
@@ -26915,7 +26962,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="462" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A462" s="6" t="s">
         <v>19</v>
       </c>
@@ -26971,7 +27018,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="463" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A463" s="6" t="s">
         <v>19</v>
       </c>
@@ -27027,7 +27074,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="464" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A464" s="6" t="s">
         <v>175</v>
       </c>
@@ -27083,7 +27130,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="465" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A465" s="6" t="s">
         <v>19</v>
       </c>
@@ -27139,7 +27186,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="466" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A466" s="6" t="s">
         <v>19</v>
       </c>
@@ -27195,7 +27242,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="467" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A467" s="6" t="s">
         <v>19</v>
       </c>
@@ -27251,7 +27298,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="468" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A468" s="6" t="s">
         <v>19</v>
       </c>
@@ -27307,7 +27354,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="469" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A469" s="6" t="s">
         <v>19</v>
       </c>
@@ -27363,7 +27410,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="470" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A470" s="6" t="s">
         <v>19</v>
       </c>
@@ -27419,7 +27466,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="471" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A471" s="6" t="s">
         <v>178</v>
       </c>
@@ -27475,7 +27522,7 @@
         <v>7.75</v>
       </c>
     </row>
-    <row r="472" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A472" s="6" t="s">
         <v>19</v>
       </c>
@@ -27531,7 +27578,7 @@
         <v>7.25</v>
       </c>
     </row>
-    <row r="473" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A473" s="6" t="s">
         <v>19</v>
       </c>
@@ -27587,7 +27634,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="474" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A474" s="6" t="s">
         <v>19</v>
       </c>
@@ -27643,7 +27690,7 @@
         <v>6.75</v>
       </c>
     </row>
-    <row r="475" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A475" s="6" t="s">
         <v>19</v>
       </c>
@@ -27699,7 +27746,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="476" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A476" s="6" t="s">
         <v>19</v>
       </c>
@@ -27755,7 +27802,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="477" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A477" s="6" t="s">
         <v>19</v>
       </c>
@@ -27811,7 +27858,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="478" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A478" s="6" t="s">
         <v>19</v>
       </c>
@@ -27867,7 +27914,7 @@
         <v>37.75</v>
       </c>
     </row>
-    <row r="479" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A479" s="6" t="s">
         <v>180</v>
       </c>
@@ -27923,7 +27970,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="480" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A480" s="6" t="s">
         <v>19</v>
       </c>
@@ -27979,7 +28026,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="481" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A481" s="6" t="s">
         <v>19</v>
       </c>
@@ -28035,7 +28082,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="482" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A482" s="6" t="s">
         <v>19</v>
       </c>
@@ -28091,7 +28138,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="483" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A483" s="6" t="s">
         <v>19</v>
       </c>
@@ -28147,7 +28194,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="484" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A484" s="6" t="s">
         <v>19</v>
       </c>
@@ -28203,7 +28250,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="485" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A485" s="6" t="s">
         <v>19</v>
       </c>
@@ -28259,7 +28306,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="486" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:18" ht="12" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A486" s="14" t="s">
         <v>182</v>
       </c>
@@ -28313,6 +28360,337 @@
       </c>
       <c r="R486" s="17">
         <v>1787.75</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8DE2F2D-0EB8-4057-AAD9-CD46211822C5}">
+  <dimension ref="B3:B66"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B3" t="str" cm="1">
+        <f t="array" ref="B3:B66">_xlfn._xlws.SORT(_xlfn.UNIQUE(sheet!D2:D1000))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B4" t="str">
+        <v>Babinecz Narcisa Bianca</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B5" t="str">
+        <v>Baciu Dumitru</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B6" t="str">
+        <v>Baran Marcin</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B7" t="str">
+        <v>Bernad Maciej</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B8" t="str">
+        <v>Bodykto Kamila Nikola</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B9" t="str">
+        <v>Browarski Marcin</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B10" t="str">
+        <v>Cotrau Mircea</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B11" t="str">
+        <v>Czenczek Mateusz</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B12" t="str">
+        <v>Da Silva Coelho Stephen Ricardo</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B13" t="str">
+        <v>Da Silva Figueiredo Laura Alexandra</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B14" t="str">
+        <v>Dudek Bartosz</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B15" t="str">
+        <v>Firlej Ryszard</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B16" t="str">
+        <v>Franczok Andrzej</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B17" t="str">
+        <v>Gagaitis Karolis</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B18" t="str">
+        <v>Gryglik Katarzyna</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B19" t="str">
+        <v>Guilherme Victorino</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B20" t="str">
+        <v>Hagiu Elena Cristina</v>
+      </c>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B21" t="str">
+        <v>Imbrowicz Ewa</v>
+      </c>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B22" t="str">
+        <v>Jaworska Justyna</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B23" t="str">
+        <v>Jozwiak Mariusz</v>
+      </c>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B24" t="str">
+        <v>Kaczmarczyk Renata</v>
+      </c>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B25" t="str">
+        <v>Katana Katarzyna</v>
+      </c>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B26" t="str">
+        <v>Kedzior Ewa</v>
+      </c>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B27" t="str">
+        <v>Kolacz Marcin</v>
+      </c>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B28" t="str">
+        <v>Kowalkowski Dominik Janusz</v>
+      </c>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B29" t="str">
+        <v>Koza Lukasz</v>
+      </c>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B30" t="str">
+        <v>Lemezonaite Evelina</v>
+      </c>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B31" t="str">
+        <v>Lisiewicz Jaroslaw</v>
+      </c>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B32" t="str">
+        <v>Marks 15815796 Pawel</v>
+      </c>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B33" t="str">
+        <v>Mihai Mihaela-Catalina</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B34" t="str">
+        <v>Minta Anna</v>
+      </c>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B35" t="str">
+        <v>Miszcak Anika Nicola</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B36" t="str">
+        <v>Mziray Salimini</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B37" t="str">
+        <v>Nilsson Jonas Sven Roger</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B38" t="str">
+        <v>Nowakowski Lukasz</v>
+      </c>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B39" t="str">
+        <v xml:space="preserve">Petrachiuta  David </v>
+      </c>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B40" t="str">
+        <v>Pluta Beata</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B41" t="str">
+        <v>Pokrajac Sasa</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B42" t="str">
+        <v>Pyttel Dawid</v>
+      </c>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B43" t="str">
+        <v>Raduszewski Marcin</v>
+      </c>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B44" t="str">
+        <v>Roman Patrik</v>
+      </c>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B45" t="str">
+        <v>Ruszkowska Anna Magdalena</v>
+      </c>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B46" t="str">
+        <v>Savicius Dominykas</v>
+      </c>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B47" t="str">
+        <v>Skrzypiec Kamil</v>
+      </c>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B48" t="str">
+        <v>Slawik Karolina</v>
+      </c>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B49" t="str">
+        <v>Stanionis Griedrius</v>
+      </c>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B50" t="str">
+        <v>Stefan Jakub</v>
+      </c>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B51" t="str">
+        <v>Stepien Szczepan</v>
+      </c>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B52" t="str">
+        <v>Stormowski Blazej Przemyslaw</v>
+      </c>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B53" t="str">
+        <v>Tanase Boris Andrei</v>
+      </c>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B54" t="str">
+        <v xml:space="preserve">Tanase Ionut-Gabriel </v>
+      </c>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B55" t="str">
+        <v>Tekiela  Natalia</v>
+      </c>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B56" t="str">
+        <v>Tol Stefan Bogdan</v>
+      </c>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B57" t="str">
+        <v>Trumpis Haris</v>
+      </c>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B58" t="str">
+        <v>Ungureanu Florica</v>
+      </c>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B59" t="str">
+        <v>Ungureanu Lenuta</v>
+      </c>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B60" t="str">
+        <v>Vaselis Jonas</v>
+      </c>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B61" t="str">
+        <v>Wieleba Krystian</v>
+      </c>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B62" t="str">
+        <v>Wigorenko Marcin</v>
+      </c>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B63" t="str">
+        <v>Wiktorowicz Adrian</v>
+      </c>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B64" t="str">
+        <v>Wilk Sebastian</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B65" t="str">
+        <v>Wypych Piotr</v>
+      </c>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.45">
+      <c r="B66">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -28321,6 +28699,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100266DDB54D3BF0E4381D035FE81726D55" ma:contentTypeVersion="16" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="7d949b307f139f9e44f4a17d6d560d65">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f3e24b04-d356-44d5-9eb5-201cfa4fc256" xmlns:ns3="bf41cf06-3f38-47d2-b3db-ee42d871b2cc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="21cf75cc06907f1d4573783b2880f0ac" ns2:_="" ns3:_="">
     <xsd:import namespace="f3e24b04-d356-44d5-9eb5-201cfa4fc256"/>
@@ -28563,15 +28950,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -28585,13 +28963,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69CBF4F5-640D-42C3-9EE8-B7BDC6CDD81B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38784A92-2D10-4BD1-83BA-6F6F16AE4A74}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38784A92-2D10-4BD1-83BA-6F6F16AE4A74}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{69CBF4F5-640D-42C3-9EE8-B7BDC6CDD81B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f3e24b04-d356-44d5-9eb5-201cfa4fc256"/>
+    <ds:schemaRef ds:uri="bf41cf06-3f38-47d2-b3db-ee42d871b2cc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0662EB87-9E6B-4C40-9F15-7D385EE5FEB4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0662EB87-9E6B-4C40-9F15-7D385EE5FEB4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bf41cf06-3f38-47d2-b3db-ee42d871b2cc"/>
+    <ds:schemaRef ds:uri="f3e24b04-d356-44d5-9eb5-201cfa4fc256"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>